<commit_message>
make risers and some scope mounts free
makes a lot of risers free, mostly pic rail risers and pistol mount risers, but also select optics (vudu, compm4/compm2)

- the ergo cost of the compm2 is now 0. as a result this leads to the compm2 getting 1 extra ergo for most setups. this wasn't changed because the compm4 is 1 ergo in most cases anyways
- the ergo cost for vudu mounts also became free. to compensate the vudu's ergo has gone from -5 -> -6. this should serve as a (minor) buff and a nerf for the vudu's worst and best mounts respectively. that one thing for the aug got buffed as well
</commit_message>
<xml_diff>
--- a/changes/aug-stuff.xlsx
+++ b/changes/aug-stuff.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lingl\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E81F254-1020-493F-BDF0-5606AFEFC678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24726F8F-C2DF-4E2C-9CF6-F79A218B3C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aug-stuff" sheetId="1" r:id="rId1"/>
@@ -838,9 +838,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -878,7 +878,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -984,7 +984,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1126,7 +1126,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1754,7 +1754,7 @@
         <v>-4.2</v>
       </c>
       <c r="P16">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="Q16">
         <v>0.15</v>
@@ -1770,11 +1770,11 @@
       </c>
       <c r="AA16">
         <f t="shared" si="1"/>
-        <v>-5.4</v>
+        <v>-4.4000000000000004</v>
       </c>
       <c r="AC16">
         <f t="shared" si="2"/>
-        <v>-3.0000000000000004</v>
+        <v>-2.0000000000000004</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.25">

</xml_diff>